<commit_message>
Game snake evaluations sub smell type added.
</commit_message>
<xml_diff>
--- a/evaluations/GPT/2025-03-31_103806/snake/all_smells_01/evaluation.xlsx
+++ b/evaluations/GPT/2025-03-31_103806/snake/all_smells_01/evaluation.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -19,6 +19,9 @@
     <t>Smell Type</t>
   </si>
   <si>
+    <t>Smell Sub-type</t>
+  </si>
+  <si>
     <t>Completeness</t>
   </si>
   <si>
@@ -43,21 +46,42 @@
     <t>syntactic</t>
   </si>
   <si>
+    <t>negative</t>
+  </si>
+  <si>
+    <t>passive_voice</t>
+  </si>
+  <si>
     <t>2.5.1</t>
   </si>
   <si>
     <t>lexical</t>
   </si>
   <si>
+    <t>subjective_language</t>
+  </si>
+  <si>
     <t>1.3, 1.6.1</t>
   </si>
   <si>
+    <t>vague_pronouns</t>
+  </si>
+  <si>
     <t>1.6.1</t>
   </si>
   <si>
+    <t>weak_verbs</t>
+  </si>
+  <si>
     <t>semantic</t>
   </si>
   <si>
+    <t>ambiguities</t>
+  </si>
+  <si>
+    <t>numerical_discrepancies</t>
+  </si>
+  <si>
     <t>2.3.1</t>
   </si>
   <si>
@@ -68,6 +92,12 @@
   </si>
   <si>
     <t>2.5.1, 2.5.3</t>
+  </si>
+  <si>
+    <t>optional_parts</t>
+  </si>
+  <si>
+    <t>logical_inconsistencies</t>
   </si>
   <si>
     <t>1.5.2</t>
@@ -83,7 +113,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -94,6 +124,10 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -110,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -120,8 +154,14 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -336,13 +376,14 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="15.13"/>
-    <col customWidth="1" min="4" max="4" width="31.38"/>
-    <col customWidth="1" min="5" max="5" width="15.13"/>
-    <col customWidth="1" min="6" max="6" width="31.38"/>
-    <col customWidth="1" min="7" max="7" width="18.5"/>
-    <col customWidth="1" min="8" max="8" width="17.0"/>
-    <col customWidth="1" min="9" max="10" width="15.38"/>
+    <col customWidth="1" min="3" max="3" width="20.0"/>
+    <col customWidth="1" min="4" max="4" width="15.13"/>
+    <col customWidth="1" min="5" max="5" width="31.38"/>
+    <col customWidth="1" min="6" max="6" width="15.13"/>
+    <col customWidth="1" min="7" max="7" width="31.38"/>
+    <col customWidth="1" min="8" max="8" width="18.5"/>
+    <col customWidth="1" min="9" max="9" width="17.0"/>
+    <col customWidth="1" min="10" max="11" width="15.38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -364,436 +405,486 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1"/>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="1">
         <v>1.0</v>
       </c>
       <c r="B2" s="1"/>
-      <c r="C2" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G2" s="2"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
     </row>
     <row r="3">
       <c r="A3" s="1">
         <v>2.0</v>
       </c>
       <c r="B3" s="1"/>
-      <c r="C3" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="1">
         <v>3.0</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F4" s="3"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1.0</v>
+      </c>
       <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
     </row>
     <row r="5">
       <c r="A5" s="1">
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F5" s="3"/>
+        <v>10</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="1">
+        <v>1.0</v>
+      </c>
       <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
     </row>
     <row r="6">
       <c r="A6" s="1">
         <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="F6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
+      <c r="C6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
     </row>
     <row r="7">
       <c r="A7" s="1">
         <v>6.0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F7" s="3"/>
+        <v>14</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1.0</v>
+      </c>
       <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
     </row>
     <row r="8">
       <c r="A8" s="1">
         <v>7.0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F8" s="3"/>
+        <v>10</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1.0</v>
+      </c>
       <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
     </row>
     <row r="9">
       <c r="A9" s="1">
         <v>8.0</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F9" s="3"/>
+        <v>14</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1.0</v>
+      </c>
       <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
     </row>
     <row r="10">
       <c r="A10" s="1">
         <v>9.0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F10" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1.0</v>
+      </c>
       <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
     </row>
     <row r="11">
       <c r="A11" s="1">
         <v>10.0</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
     </row>
     <row r="12">
       <c r="A12" s="1">
         <v>11.0</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F12" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1.0</v>
+      </c>
       <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
     </row>
     <row r="13">
       <c r="A13" s="1">
         <v>12.0</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+        <v>14</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
     </row>
     <row r="14">
       <c r="A14" s="1">
         <v>13.0</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+        <v>14</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
     </row>
     <row r="15">
       <c r="A15" s="1">
         <v>14.0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="F15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
+      <c r="C15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1"/>
-      <c r="C16" s="3">
-        <f>SUM(C2:C15)</f>
+      <c r="C16" s="1"/>
+      <c r="D16" s="4">
+        <f>SUM(D2:D15)</f>
         <v>4</v>
       </c>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3">
-        <f>SUM(E2:E15)</f>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4">
+        <f>SUM(F2:F15)</f>
         <v>8</v>
       </c>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
     </row>
     <row r="17">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
     </row>
     <row r="18">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
     </row>
     <row r="19">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
     </row>
     <row r="20">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
     </row>
     <row r="21">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
     </row>
     <row r="22">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
     </row>
     <row r="23">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
     </row>
     <row r="24">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
     </row>
     <row r="25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
     </row>
     <row r="26">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
     </row>
     <row r="27">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>